<commit_message>
Budget product p-gsb-001: build, listing, photos, tech and clone checks
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012TgDhDPhYU8Na94rpjNyB3
</commit_message>
<xml_diff>
--- a/data/products/p-gsb-001/work/Clear-Budget.xlsx
+++ b/data/products/p-gsb-001/work/Clear-Budget.xlsx
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="576" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="578" uniqueCount="171">
   <si>
     <t xml:space="preserve">Clear Budget</t>
   </si>
@@ -393,6 +393,9 @@
   </si>
   <si>
     <t xml:space="preserve">Card payment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Concert tickets</t>
   </si>
   <si>
     <t xml:space="preserve">Shoes</t>
@@ -1305,7 +1308,7 @@
                 <c:formatCode>\$#,##0.00;[RED]"-$"#,##0.00;\$0.00</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>1992.09</c:v>
+                  <c:v>2112.09</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1313,11 +1316,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="17068865"/>
-        <c:axId val="64864604"/>
+        <c:axId val="88460589"/>
+        <c:axId val="3627449"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="17068865"/>
+        <c:axId val="88460589"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1349,7 +1352,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="64864604"/>
+        <c:crossAx val="3627449"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1357,7 +1360,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="64864604"/>
+        <c:axId val="3627449"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1399,7 +1402,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="17068865"/>
+        <c:crossAx val="88460589"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1716,7 +1719,7 @@
                   <c:v>1523.6</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>118.49</c:v>
+                  <c:v>238.49</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>200</c:v>
@@ -2403,11 +2406,11 @@
         <v>42</v>
       </c>
       <c r="D19" s="12" t="str">
-        <f aca="false">IF(SUMPRODUCT(COUNTIF(January!$C$7:$C$86,{"Rent","Weekly shop","Bus pass","Pizza night","Weekly shop","Phone bill","To emergency fund","Streaming","Card payment","Shoes"}))=0,"Done","To do")</f>
+        <f aca="false">IF(SUMPRODUCT(COUNTIF(January!$C$7:$C$86,{"Rent","Weekly shop","Bus pass","Pizza night","Weekly shop","Phone bill","To emergency fund","Streaming","Card payment","Concert tickets","Shoes"}))=0,"Done","To do")</f>
         <v>To do</v>
       </c>
       <c r="E19" s="13" t="str">
-        <f aca="false">IF(SUMPRODUCT(COUNTIF(January!$C$7:$C$86,{"Rent","Weekly shop","Bus pass","Pizza night","Weekly shop","Phone bill","To emergency fund","Streaming","Card payment","Shoes"}))=0,"","Clear the example in January (step 2)")</f>
+        <f aca="false">IF(SUMPRODUCT(COUNTIF(January!$C$7:$C$86,{"Rent","Weekly shop","Bus pass","Pizza night","Weekly shop","Phone bill","To emergency fund","Streaming","Card payment","Concert tickets","Shoes"}))=0,"","Clear the example in January (step 2)")</f>
         <v>Clear the example in January (step 2)</v>
       </c>
     </row>
@@ -3805,7 +3808,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D4141AB6-1346-49BA-88EF-96A0ECAA648A}</x14:id>
+          <x14:id>{E07D84EA-FA2A-4CFE-8F93-B02BF890A21B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -3837,7 +3840,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D4141AB6-1346-49BA-88EF-96A0ECAA648A}">
+          <x14:cfRule type="dataBar" id="{E07D84EA-FA2A-4CFE-8F93-B02BF890A21B}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -5073,7 +5076,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{107B60FF-175B-4A7A-AE86-1063556FD2F5}</x14:id>
+          <x14:id>{A4C39EEF-21A2-4BBE-B370-BAD8FB4D942F}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -5105,7 +5108,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{107B60FF-175B-4A7A-AE86-1063556FD2F5}">
+          <x14:cfRule type="dataBar" id="{A4C39EEF-21A2-4BBE-B370-BAD8FB4D942F}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -6341,7 +6344,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{B8C56F60-D546-4C43-8A7E-7DB260E724C4}</x14:id>
+          <x14:id>{BEB9C0B4-EFE2-459E-BEB2-EFC1EA4C87AE}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -6373,7 +6376,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{B8C56F60-D546-4C43-8A7E-7DB260E724C4}">
+          <x14:cfRule type="dataBar" id="{BEB9C0B4-EFE2-459E-BEB2-EFC1EA4C87AE}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -7609,7 +7612,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3CF4652D-DCE0-4D97-B29A-325E8922BDAC}</x14:id>
+          <x14:id>{D93D6873-F82E-4AD4-A244-F9D21B99BB70}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -7641,7 +7644,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3CF4652D-DCE0-4D97-B29A-325E8922BDAC}">
+          <x14:cfRule type="dataBar" id="{D93D6873-F82E-4AD4-A244-F9D21B99BB70}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -8877,7 +8880,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3323BD54-9920-4662-A570-C84899F0C48B}</x14:id>
+          <x14:id>{8C34BB72-D0CD-4820-89E3-E85F4642F596}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -8909,7 +8912,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3323BD54-9920-4662-A570-C84899F0C48B}">
+          <x14:cfRule type="dataBar" id="{8C34BB72-D0CD-4820-89E3-E85F4642F596}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -10145,7 +10148,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{84764CE0-206A-4C32-9D7D-187D244B5915}</x14:id>
+          <x14:id>{14A17C10-FAA2-47F9-A079-A15C71B0572E}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10177,7 +10180,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{84764CE0-206A-4C32-9D7D-187D244B5915}">
+          <x14:cfRule type="dataBar" id="{14A17C10-FAA2-47F9-A079-A15C71B0572E}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -10221,7 +10224,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10252,52 +10255,52 @@
     </row>
     <row r="6" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="10" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D6" s="10" t="s">
         <v>102</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F6" s="10" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="H6" s="10" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="J6" s="10" t="s">
         <v>24</v>
       </c>
       <c r="K6" s="10" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="L6" s="10" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="M6" s="10" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="N6" s="10" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="O6" s="10" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="P6" s="10" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="Q6" s="10" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10311,7 +10314,7 @@
         <v>1400</v>
       </c>
       <c r="E7" s="17" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F7" s="34"/>
       <c r="G7" s="34"/>
@@ -10337,7 +10340,7 @@
         <v>95</v>
       </c>
       <c r="E8" s="17" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F8" s="34"/>
       <c r="G8" s="34"/>
@@ -10363,7 +10366,7 @@
         <v>15.99</v>
       </c>
       <c r="E9" s="17" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F9" s="34"/>
       <c r="G9" s="34"/>
@@ -10380,7 +10383,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="17" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C10" s="25" t="n">
         <v>20</v>
@@ -10389,7 +10392,7 @@
         <v>160</v>
       </c>
       <c r="E10" s="17" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F10" s="34"/>
       <c r="G10" s="34"/>
@@ -10406,7 +10409,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="17" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C11" s="25" t="n">
         <v>22</v>
@@ -10415,7 +10418,7 @@
         <v>90</v>
       </c>
       <c r="E11" s="17" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F11" s="34"/>
       <c r="G11" s="34"/>
@@ -10441,7 +10444,7 @@
         <v>150</v>
       </c>
       <c r="E12" s="17" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F12" s="34"/>
       <c r="G12" s="34"/>
@@ -10800,7 +10803,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="19" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D32" s="23" t="n">
         <f aca="false">SUM(D7:D31)</f>
@@ -10856,12 +10859,12 @@
   <sheetData>
     <row r="2" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10892,7 +10895,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="19" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C6" s="35" t="n">
         <f aca="false">DATE(Year,1,1)+MOD(6-WEEKDAY(DATE(Year,1,1)),7)</f>
@@ -10901,39 +10904,39 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="19" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="19" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C8" s="26" t="n">
         <f aca="false">ROUND(Setup!$C$10*12/CHOOSE(MATCH($C$7,{"Weekly","Every 2 weeks","Twice a month","Monthly"},0),52,26,24,12),2)</f>
         <v>1661.54</v>
       </c>
       <c r="D8" s="29" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="10" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C10" s="10" t="s">
         <v>7</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F10" s="10" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11583,12 +11586,12 @@
   <sheetData>
     <row r="2" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="1" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="2" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11619,15 +11622,15 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="19" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C7" s="26" t="n">
         <v>100</v>
@@ -11638,22 +11641,22 @@
         <v>8</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="F9" s="10" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="G9" s="10" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="H9" s="10" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11684,7 +11687,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="17" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C11" s="26" t="n">
         <v>8200</v>
@@ -11862,7 +11865,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="19" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C20" s="23" t="n">
         <f aca="false">SUM(C10:C19)</f>
@@ -11920,12 +11923,12 @@
   <sheetData>
     <row r="2" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="1" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="2" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11956,22 +11959,22 @@
     </row>
     <row r="6" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="10" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D6" s="10" t="s">
         <v>63</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F6" s="10" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11998,7 +12001,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="17" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C8" s="26" t="n">
         <v>1800</v>
@@ -12020,7 +12023,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="17" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C9" s="26" t="n">
         <v>1200</v>
@@ -12149,7 +12152,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C39A6DE7-83A0-48D5-B57E-CC933EB7C91B}</x14:id>
+          <x14:id>{71AA7A77-EAB6-45C0-BFD0-BEE8AC647617}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -12175,7 +12178,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C39A6DE7-83A0-48D5-B57E-CC933EB7C91B}">
+          <x14:cfRule type="dataBar" id="{71AA7A77-EAB6-45C0-BFD0-BEE8AC647617}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -12280,11 +12283,11 @@
       </c>
       <c r="D7" s="22" t="n">
         <f aca="false">IF(COUNT(January!$E$7:$E$86)&gt;0,January!H7,"")</f>
-        <v>1992.09</v>
+        <v>2112.09</v>
       </c>
       <c r="E7" s="22" t="n">
         <f aca="false">IF(COUNT(January!$E$7:$E$86)&gt;0,January!H8,"")</f>
-        <v>1907.91</v>
+        <v>1787.91</v>
       </c>
       <c r="F7" s="22" t="n">
         <f aca="false">IF(COUNT(January!$E$7:$E$86)&gt;0,January!H9,"")</f>
@@ -12626,7 +12629,7 @@
       </c>
       <c r="I17" s="22" t="n">
         <f aca="false">IF(H17="","",SUMIFS(January!$E$7:$E$86,January!$D$7:$D$86,H17)+SUMIFS(February!$E$7:$E$86,February!$D$7:$D$86,H17)+SUMIFS(March!$E$7:$E$86,March!$D$7:$D$86,H17)+SUMIFS(April!$E$7:$E$86,April!$D$7:$D$86,H17)+SUMIFS(May!$E$7:$E$86,May!$D$7:$D$86,H17)+SUMIFS(June!$E$7:$E$86,June!$D$7:$D$86,H17)+SUMIFS(July!$E$7:$E$86,July!$D$7:$D$86,H17)+SUMIFS(August!$E$7:$E$86,August!$D$7:$D$86,H17)+SUMIFS(September!$E$7:$E$86,September!$D$7:$D$86,H17)+SUMIFS(October!$E$7:$E$86,October!$D$7:$D$86,H17)+SUMIFS(November!$E$7:$E$86,November!$D$7:$D$86,H17)+SUMIFS(December!$E$7:$E$86,December!$D$7:$D$86,H17))</f>
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="J17" s="11" t="str">
         <f aca="false">IF(H17="","",Setup!F20)</f>
@@ -12676,11 +12679,11 @@
       </c>
       <c r="D19" s="23" t="n">
         <f aca="false">SUM(D7:D18)</f>
-        <v>1992.09</v>
+        <v>2112.09</v>
       </c>
       <c r="E19" s="23" t="n">
         <f aca="false">SUM(E7:E18)</f>
-        <v>1907.91</v>
+        <v>1787.91</v>
       </c>
       <c r="F19" s="23" t="n">
         <f aca="false">SUM(F7:F18)</f>
@@ -12795,7 +12798,7 @@
       </c>
       <c r="C25" s="22" t="n">
         <f aca="false">SUMIF($J$7:$J$36,"Wants",$I$7:$I$36)</f>
-        <v>118.49</v>
+        <v>238.49</v>
       </c>
       <c r="H25" s="11" t="str">
         <f aca="false">IF(Setup!E28="","",Setup!E28)</f>
@@ -13537,7 +13540,7 @@
       </c>
       <c r="H7" s="32" t="n">
         <f aca="false">SUM(E7:E86)</f>
-        <v>1992.09</v>
+        <v>2112.09</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13558,7 +13561,7 @@
       </c>
       <c r="H8" s="32" t="n">
         <f aca="false">H6-H7</f>
-        <v>1907.91</v>
+        <v>1787.91</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13763,16 +13766,16 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="30" t="n">
-        <v>46412</v>
+        <v>46411</v>
       </c>
       <c r="C16" s="17" t="s">
         <v>117</v>
       </c>
       <c r="D16" s="17" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E16" s="26" t="n">
-        <v>64</v>
+        <v>120</v>
       </c>
       <c r="G16" s="11" t="str">
         <f aca="false">IF(Setup!E14="","",Setup!E14)</f>
@@ -13796,10 +13799,18 @@
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="30"/>
-      <c r="C17" s="17"/>
-      <c r="D17" s="17"/>
-      <c r="E17" s="26"/>
+      <c r="B17" s="30" t="n">
+        <v>46412</v>
+      </c>
+      <c r="C17" s="17" t="s">
+        <v>118</v>
+      </c>
+      <c r="D17" s="17" t="s">
+        <v>87</v>
+      </c>
+      <c r="E17" s="26" t="n">
+        <v>64</v>
+      </c>
       <c r="G17" s="11" t="str">
         <f aca="false">IF(Setup!E15="","",Setup!E15)</f>
         <v>Phone and internet</v>
@@ -13940,15 +13951,15 @@
       </c>
       <c r="I22" s="22" t="n">
         <f aca="false">IF(G22="","",SUMIFS($E$7:$E$86,$D$7:$D$86,G22))</f>
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="J22" s="22" t="n">
         <f aca="false">IF(G22="","",H22-I22)</f>
-        <v>100</v>
+        <v>-20</v>
       </c>
       <c r="K22" s="33" t="n">
         <f aca="false">IF(OR(G22="",H22=0),"",I22/H22)</f>
-        <v>0</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14736,7 +14747,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{9951EF64-182C-43EA-93C8-2CDA19405FB7}</x14:id>
+          <x14:id>{74F8BB22-BC17-49AD-9A67-46D4F496E72D}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -14768,7 +14779,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{9951EF64-182C-43EA-93C8-2CDA19405FB7}">
+          <x14:cfRule type="dataBar" id="{74F8BB22-BC17-49AD-9A67-46D4F496E72D}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -16004,7 +16015,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C4CDDC1B-47FE-4291-A3FB-4795DDE5EAC1}</x14:id>
+          <x14:id>{458F88EA-3D7B-4982-92C3-893F97DDDDD7}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -16036,7 +16047,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C4CDDC1B-47FE-4291-A3FB-4795DDE5EAC1}">
+          <x14:cfRule type="dataBar" id="{458F88EA-3D7B-4982-92C3-893F97DDDDD7}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -17272,7 +17283,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{AAC6B72D-3A36-4E98-8E81-88DAEB84F727}</x14:id>
+          <x14:id>{708998E1-C340-47E1-B449-9D5344B5571A}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -17304,7 +17315,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{AAC6B72D-3A36-4E98-8E81-88DAEB84F727}">
+          <x14:cfRule type="dataBar" id="{708998E1-C340-47E1-B449-9D5344B5571A}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -18540,7 +18551,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F76153D5-9DA1-4AFE-9620-F0AF2B1060FF}</x14:id>
+          <x14:id>{17C03557-6C50-4D2A-83E9-D795DD98C91F}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -18572,7 +18583,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F76153D5-9DA1-4AFE-9620-F0AF2B1060FF}">
+          <x14:cfRule type="dataBar" id="{17C03557-6C50-4D2A-83E9-D795DD98C91F}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -19808,7 +19819,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{8C6C3A85-446B-4319-93FE-9846F5EF501A}</x14:id>
+          <x14:id>{C0651B90-5B3A-49A3-9E64-3EE0724EB62B}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -19840,7 +19851,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{8C6C3A85-446B-4319-93FE-9846F5EF501A}">
+          <x14:cfRule type="dataBar" id="{C0651B90-5B3A-49A3-9E64-3EE0724EB62B}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -21076,7 +21087,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F9D37BED-4064-48B4-8A7A-787CC08DC397}</x14:id>
+          <x14:id>{25F41094-89EE-4AEE-AE4B-93C95B4B2014}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -21108,7 +21119,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F9D37BED-4064-48B4-8A7A-787CC08DC397}">
+          <x14:cfRule type="dataBar" id="{25F41094-89EE-4AEE-AE4B-93C95B4B2014}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>

</xml_diff>

<commit_message>
Clear Budget: listing revised, unique photo crops, round 2 check prepared
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012TgDhDPhYU8Na94rpjNyB3
</commit_message>
<xml_diff>
--- a/data/products/p-gsb-001/work/Clear-Budget.xlsx
+++ b/data/products/p-gsb-001/work/Clear-Budget.xlsx
@@ -1333,11 +1333,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="45720845"/>
-        <c:axId val="67391242"/>
+        <c:axId val="62159819"/>
+        <c:axId val="60585776"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="45720845"/>
+        <c:axId val="62159819"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1369,7 +1369,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="67391242"/>
+        <c:crossAx val="60585776"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1377,7 +1377,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="67391242"/>
+        <c:axId val="60585776"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1419,7 +1419,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="45720845"/>
+        <c:crossAx val="62159819"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1808,8 +1808,8 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>684720</xdr:colOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>1037160</xdr:colOff>
       <xdr:row>50</xdr:row>
       <xdr:rowOff>32760</xdr:rowOff>
     </xdr:to>
@@ -1839,7 +1839,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>858600</xdr:colOff>
+      <xdr:colOff>858240</xdr:colOff>
       <xdr:row>33</xdr:row>
       <xdr:rowOff>175320</xdr:rowOff>
     </xdr:to>
@@ -1849,7 +1849,7 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="2185200" y="4324320"/>
+        <a:off x="2960280" y="4324320"/>
         <a:ext cx="3959640" cy="2699640"/>
       </xdr:xfrm>
       <a:graphic>
@@ -13460,7 +13460,8 @@
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="0" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="24"/>

</xml_diff>

<commit_message>
Clear Budget passed check round 3, queued for review
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012TgDhDPhYU8Na94rpjNyB3
</commit_message>
<xml_diff>
--- a/data/products/p-gsb-001/work/Clear-Budget.xlsx
+++ b/data/products/p-gsb-001/work/Clear-Budget.xlsx
@@ -533,7 +533,7 @@
     <t xml:space="preserve">Interest saved</t>
   </si>
   <si>
-    <t xml:space="preserve">Medical bill</t>
+    <t xml:space="preserve">Store card</t>
   </si>
   <si>
     <t xml:space="preserve">Car loan</t>
@@ -1347,11 +1347,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="31805084"/>
-        <c:axId val="59715233"/>
+        <c:axId val="26444737"/>
+        <c:axId val="45113722"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="31805084"/>
+        <c:axId val="26444737"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1383,7 +1383,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="59715233"/>
+        <c:crossAx val="45113722"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1391,7 +1391,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="59715233"/>
+        <c:axId val="45113722"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1433,7 +1433,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="31805084"/>
+        <c:crossAx val="26444737"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1853,7 +1853,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>858240</xdr:colOff>
+      <xdr:colOff>505800</xdr:colOff>
       <xdr:row>31</xdr:row>
       <xdr:rowOff>42120</xdr:rowOff>
     </xdr:to>
@@ -10920,7 +10920,7 @@
       <c r="D7" s="26" t="n">
         <v>1400</v>
       </c>
-      <c r="E7" s="17" t="s">
+      <c r="E7" s="34" t="s">
         <v>134</v>
       </c>
       <c r="F7" s="34"/>
@@ -10946,7 +10946,7 @@
       <c r="D8" s="26" t="n">
         <v>95</v>
       </c>
-      <c r="E8" s="17" t="s">
+      <c r="E8" s="34" t="s">
         <v>134</v>
       </c>
       <c r="F8" s="34"/>
@@ -10972,7 +10972,7 @@
       <c r="D9" s="26" t="n">
         <v>15.99</v>
       </c>
-      <c r="E9" s="17" t="s">
+      <c r="E9" s="34" t="s">
         <v>134</v>
       </c>
       <c r="F9" s="34"/>
@@ -10998,7 +10998,7 @@
       <c r="D10" s="26" t="n">
         <v>160</v>
       </c>
-      <c r="E10" s="17" t="s">
+      <c r="E10" s="34" t="s">
         <v>136</v>
       </c>
       <c r="F10" s="34"/>
@@ -11024,7 +11024,7 @@
       <c r="D11" s="26" t="n">
         <v>90</v>
       </c>
-      <c r="E11" s="17" t="s">
+      <c r="E11" s="34" t="s">
         <v>136</v>
       </c>
       <c r="F11" s="34"/>
@@ -11050,7 +11050,7 @@
       <c r="D12" s="26" t="n">
         <v>150</v>
       </c>
-      <c r="E12" s="17" t="s">
+      <c r="E12" s="34" t="s">
         <v>136</v>
       </c>
       <c r="F12" s="34"/>
@@ -11070,7 +11070,7 @@
       <c r="B13" s="17"/>
       <c r="C13" s="25"/>
       <c r="D13" s="26"/>
-      <c r="E13" s="17"/>
+      <c r="E13" s="34"/>
       <c r="F13" s="34"/>
       <c r="G13" s="34"/>
       <c r="H13" s="34"/>
@@ -11088,7 +11088,7 @@
       <c r="B14" s="17"/>
       <c r="C14" s="25"/>
       <c r="D14" s="26"/>
-      <c r="E14" s="17"/>
+      <c r="E14" s="34"/>
       <c r="F14" s="34"/>
       <c r="G14" s="34"/>
       <c r="H14" s="34"/>
@@ -11106,7 +11106,7 @@
       <c r="B15" s="17"/>
       <c r="C15" s="25"/>
       <c r="D15" s="26"/>
-      <c r="E15" s="17"/>
+      <c r="E15" s="34"/>
       <c r="F15" s="34"/>
       <c r="G15" s="34"/>
       <c r="H15" s="34"/>
@@ -11124,7 +11124,7 @@
       <c r="B16" s="17"/>
       <c r="C16" s="25"/>
       <c r="D16" s="26"/>
-      <c r="E16" s="17"/>
+      <c r="E16" s="34"/>
       <c r="F16" s="34"/>
       <c r="G16" s="34"/>
       <c r="H16" s="34"/>
@@ -11142,7 +11142,7 @@
       <c r="B17" s="17"/>
       <c r="C17" s="25"/>
       <c r="D17" s="26"/>
-      <c r="E17" s="17"/>
+      <c r="E17" s="34"/>
       <c r="F17" s="34"/>
       <c r="G17" s="34"/>
       <c r="H17" s="34"/>
@@ -11160,7 +11160,7 @@
       <c r="B18" s="17"/>
       <c r="C18" s="25"/>
       <c r="D18" s="26"/>
-      <c r="E18" s="17"/>
+      <c r="E18" s="34"/>
       <c r="F18" s="34"/>
       <c r="G18" s="34"/>
       <c r="H18" s="34"/>
@@ -11178,7 +11178,7 @@
       <c r="B19" s="17"/>
       <c r="C19" s="25"/>
       <c r="D19" s="26"/>
-      <c r="E19" s="17"/>
+      <c r="E19" s="34"/>
       <c r="F19" s="34"/>
       <c r="G19" s="34"/>
       <c r="H19" s="34"/>
@@ -11196,7 +11196,7 @@
       <c r="B20" s="17"/>
       <c r="C20" s="25"/>
       <c r="D20" s="26"/>
-      <c r="E20" s="17"/>
+      <c r="E20" s="34"/>
       <c r="F20" s="34"/>
       <c r="G20" s="34"/>
       <c r="H20" s="34"/>
@@ -11214,7 +11214,7 @@
       <c r="B21" s="17"/>
       <c r="C21" s="25"/>
       <c r="D21" s="26"/>
-      <c r="E21" s="17"/>
+      <c r="E21" s="34"/>
       <c r="F21" s="34"/>
       <c r="G21" s="34"/>
       <c r="H21" s="34"/>
@@ -11232,7 +11232,7 @@
       <c r="B22" s="17"/>
       <c r="C22" s="25"/>
       <c r="D22" s="26"/>
-      <c r="E22" s="17"/>
+      <c r="E22" s="34"/>
       <c r="F22" s="34"/>
       <c r="G22" s="34"/>
       <c r="H22" s="34"/>
@@ -11250,7 +11250,7 @@
       <c r="B23" s="17"/>
       <c r="C23" s="25"/>
       <c r="D23" s="26"/>
-      <c r="E23" s="17"/>
+      <c r="E23" s="34"/>
       <c r="F23" s="34"/>
       <c r="G23" s="34"/>
       <c r="H23" s="34"/>
@@ -11268,7 +11268,7 @@
       <c r="B24" s="17"/>
       <c r="C24" s="25"/>
       <c r="D24" s="26"/>
-      <c r="E24" s="17"/>
+      <c r="E24" s="34"/>
       <c r="F24" s="34"/>
       <c r="G24" s="34"/>
       <c r="H24" s="34"/>
@@ -11286,7 +11286,7 @@
       <c r="B25" s="17"/>
       <c r="C25" s="25"/>
       <c r="D25" s="26"/>
-      <c r="E25" s="17"/>
+      <c r="E25" s="34"/>
       <c r="F25" s="34"/>
       <c r="G25" s="34"/>
       <c r="H25" s="34"/>
@@ -11304,7 +11304,7 @@
       <c r="B26" s="17"/>
       <c r="C26" s="25"/>
       <c r="D26" s="26"/>
-      <c r="E26" s="17"/>
+      <c r="E26" s="34"/>
       <c r="F26" s="34"/>
       <c r="G26" s="34"/>
       <c r="H26" s="34"/>
@@ -11322,7 +11322,7 @@
       <c r="B27" s="17"/>
       <c r="C27" s="25"/>
       <c r="D27" s="26"/>
-      <c r="E27" s="17"/>
+      <c r="E27" s="34"/>
       <c r="F27" s="34"/>
       <c r="G27" s="34"/>
       <c r="H27" s="34"/>
@@ -11340,7 +11340,7 @@
       <c r="B28" s="17"/>
       <c r="C28" s="25"/>
       <c r="D28" s="26"/>
-      <c r="E28" s="17"/>
+      <c r="E28" s="34"/>
       <c r="F28" s="34"/>
       <c r="G28" s="34"/>
       <c r="H28" s="34"/>
@@ -11358,7 +11358,7 @@
       <c r="B29" s="17"/>
       <c r="C29" s="25"/>
       <c r="D29" s="26"/>
-      <c r="E29" s="17"/>
+      <c r="E29" s="34"/>
       <c r="F29" s="34"/>
       <c r="G29" s="34"/>
       <c r="H29" s="34"/>
@@ -11376,7 +11376,7 @@
       <c r="B30" s="17"/>
       <c r="C30" s="25"/>
       <c r="D30" s="26"/>
-      <c r="E30" s="17"/>
+      <c r="E30" s="34"/>
       <c r="F30" s="34"/>
       <c r="G30" s="34"/>
       <c r="H30" s="34"/>
@@ -11394,7 +11394,7 @@
       <c r="B31" s="17"/>
       <c r="C31" s="25"/>
       <c r="D31" s="26"/>
-      <c r="E31" s="17"/>
+      <c r="E31" s="34"/>
       <c r="F31" s="34"/>
       <c r="G31" s="34"/>
       <c r="H31" s="34"/>
@@ -12879,10 +12879,10 @@
         <v>600</v>
       </c>
       <c r="D10" s="38" t="n">
-        <v>0</v>
+        <v>0.1999</v>
       </c>
       <c r="E10" s="26" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="F10" s="39" t="n">
         <f aca="false">IF(C10="","",IF($C$6="Snowball",COUNTIFS($C$10:$C$19,"&lt;"&amp;C10,$C$10:$C$19,"&lt;&gt;")+1,COUNTIFS($D$10:$D$19,"&gt;"&amp;D10,$C$10:$C$19,"&lt;&gt;")+1))</f>
@@ -12890,19 +12890,19 @@
       </c>
       <c r="G10" s="39" t="n">
         <f aca="false">IF(OR(C10="",E10=""),"",IFERROR(ROUNDUP(NPER(D10/12,-E10,C10),0),"never: raise the minimum"))</f>
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="H10" s="22" t="n">
         <f aca="false">IF(OR(C10="",E10="",NOT(ISNUMBER(G10))),"",G10*E10-C10)</f>
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="I10" s="39" t="n">
         <f aca="false">IF(OR(C10="",E10="",F10&lt;&gt;1),"",IFERROR(ROUNDUP(NPER(D10/12,-(E10+$C$7),C10),0),""))</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J10" s="22" t="n">
         <f aca="false">IF(OR(I10="",NOT(ISNUMBER(H10))),"",MAX(0,H10-(I10*(E10+$C$7)-C10)))</f>
-        <v>0</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12913,7 +12913,7 @@
         <v>2400</v>
       </c>
       <c r="D11" s="38" t="n">
-        <v>0.2299</v>
+        <v>0.2499</v>
       </c>
       <c r="E11" s="26" t="n">
         <v>75</v>
@@ -12924,11 +12924,11 @@
       </c>
       <c r="G11" s="39" t="n">
         <f aca="false">IF(OR(C11="",E11=""),"",IFERROR(ROUNDUP(NPER(D11/12,-E11,C11),0),"never: raise the minimum"))</f>
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="H11" s="22" t="n">
         <f aca="false">IF(OR(C11="",E11="",NOT(ISNUMBER(G11))),"",G11*E11-C11)</f>
-        <v>1425</v>
+        <v>1650</v>
       </c>
       <c r="I11" s="39" t="str">
         <f aca="false">IF(OR(C11="",E11="",F11&lt;&gt;1),"",IFERROR(ROUNDUP(NPER(D11/12,-(E11+$C$7),C11),0),""))</f>
@@ -13173,7 +13173,7 @@
       </c>
       <c r="E20" s="23" t="n">
         <f aca="false">SUM(E10:E19)</f>
-        <v>515</v>
+        <v>505</v>
       </c>
     </row>
   </sheetData>
@@ -13517,7 +13517,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="21"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="24"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="16"/>

</xml_diff>